<commit_message>
added literature and new PDM formatting
</commit_message>
<xml_diff>
--- a/admin/Project management/Project timeline management(caa 17.10.25).xlsx
+++ b/admin/Project management/Project timeline management(caa 17.10.25).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ling Jun\Desktop\PSB\AI-ethics\admin\Project management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F031F4-6097-42D9-A15C-EC8A8C4B6C49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC42C7C-25A0-4D7A-9D56-07DB8E05DDCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-119" yWindow="-119" windowWidth="28741" windowHeight="15543" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28399" yWindow="7541" windowWidth="16241" windowHeight="13955" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt Chart (daily view)" sheetId="13" r:id="rId1"/>
@@ -125,9 +125,6 @@
     <t>https://www.vertex42.com/ExcelTemplates/task-list-template.html</t>
   </si>
   <si>
-    <t>Plan Days</t>
-  </si>
-  <si>
     <t>Get Gantt Chart Template Pro for Excel</t>
   </si>
   <si>
@@ -459,6 +456,9 @@
   </si>
   <si>
     <t>Priority</t>
+  </si>
+  <si>
+    <t>Working days</t>
   </si>
 </sst>
 </file>
@@ -681,7 +681,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="51">
     <border>
       <left/>
       <right/>
@@ -1163,6 +1163,184 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1174,7 +1352,7 @@
     </xf>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1263,25 +1441,16 @@
     <xf numFmtId="0" fontId="20" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="20" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="20" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1314,16 +1483,10 @@
     <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="20" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1337,9 +1500,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1359,37 +1519,13 @@
     <xf numFmtId="9" fontId="20" fillId="0" borderId="31" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="17" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="20" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="20" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="20" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="20" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="20" fillId="0" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1409,18 +1545,6 @@
     </xf>
     <xf numFmtId="1" fontId="20" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1449,34 +1573,88 @@
     <xf numFmtId="14" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="20" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="20" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="20" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="20" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill>
@@ -1581,15 +1759,15 @@
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{2073864A-197E-4405-AEEA-612BC929274A}"/>
     <tableStyle name="ToDoList" pivot="0" count="9" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="12"/>
-      <tableStyleElement type="headerRow" dxfId="11"/>
-      <tableStyleElement type="totalRow" dxfId="10"/>
-      <tableStyleElement type="firstColumn" dxfId="9"/>
-      <tableStyleElement type="lastColumn" dxfId="8"/>
-      <tableStyleElement type="firstRowStripe" dxfId="7"/>
-      <tableStyleElement type="secondRowStripe" dxfId="6"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="5"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="4"/>
+      <tableStyleElement type="wholeTable" dxfId="9"/>
+      <tableStyleElement type="headerRow" dxfId="8"/>
+      <tableStyleElement type="totalRow" dxfId="7"/>
+      <tableStyleElement type="firstColumn" dxfId="6"/>
+      <tableStyleElement type="lastColumn" dxfId="5"/>
+      <tableStyleElement type="firstRowStripe" dxfId="4"/>
+      <tableStyleElement type="secondRowStripe" dxfId="3"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="2"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -2075,13 +2253,13 @@
                   <c:v>56</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>90</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>99</c:v>
+                  <c:v>67</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>104</c:v>
+                  <c:v>73</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>125</c:v>
@@ -2123,7 +2301,7 @@
                   <c:v>38</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>38</c:v>
+                  <c:v>281</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2276,19 +2454,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="26"/>
                 <c:pt idx="0">
-                  <c:v>13</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10.5</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.1</c:v>
+                  <c:v>1.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>10</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -2507,10 +2685,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10.5</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18.899999999999999</c:v>
+                  <c:v>13.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -2519,64 +2697,64 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>11</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>7</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>44</c:v>
-                </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="18">
                   <c:v>9</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="19">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="21">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="12">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>21</c:v>
-                </c:pt>
                 <c:pt idx="22">
-                  <c:v>20</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="23">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>244</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3545,13 +3723,13 @@
                   <c:v>56</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>90</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>99</c:v>
+                  <c:v>67</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>104</c:v>
+                  <c:v>73</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>125</c:v>
@@ -3593,7 +3771,7 @@
                   <c:v>38</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>38</c:v>
+                  <c:v>281</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3746,19 +3924,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="26"/>
                 <c:pt idx="0">
-                  <c:v>13</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10.5</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.1</c:v>
+                  <c:v>1.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>10</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -3977,10 +4155,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10.5</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18.899999999999999</c:v>
+                  <c:v>13.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3989,64 +4167,64 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>11</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>7</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>44</c:v>
-                </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="18">
                   <c:v>9</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="19">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="21">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="12">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>21</c:v>
-                </c:pt>
                 <c:pt idx="22">
-                  <c:v>20</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="23">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>244</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5025,13 +5203,13 @@
                   <c:v>56</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>90</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>99</c:v>
+                  <c:v>67</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>104</c:v>
+                  <c:v>73</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>125</c:v>
@@ -5073,7 +5251,7 @@
                   <c:v>38</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>38</c:v>
+                  <c:v>281</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5226,19 +5404,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="26"/>
                 <c:pt idx="0">
-                  <c:v>13</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10.5</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.1</c:v>
+                  <c:v>1.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>10</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -5457,10 +5635,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10.5</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18.899999999999999</c:v>
+                  <c:v>13.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -5469,64 +5647,64 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>11</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>7</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>44</c:v>
-                </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="18">
                   <c:v>9</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="19">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="21">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="12">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>21</c:v>
-                </c:pt>
                 <c:pt idx="22">
-                  <c:v>20</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="23">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>244</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8186,7 +8364,7 @@
   <sheetData>
     <row r="1" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="6:6" x14ac:dyDescent="0.2">
@@ -8337,7 +8515,7 @@
   <sheetData>
     <row r="1" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="6:6" x14ac:dyDescent="0.2">
@@ -8488,7 +8666,7 @@
   <sheetData>
     <row r="1" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="6:6" x14ac:dyDescent="0.2">
@@ -8638,25 +8816,25 @@
   <sheetFormatPr defaultRowHeight="45.3" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="255.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="181.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.125" style="81" customWidth="1"/>
-    <col min="4" max="4" width="35.625" style="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="181.875" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="40.125" style="67" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="35.625" style="13" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="35.625" customWidth="1"/>
-    <col min="6" max="6" width="42.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.625" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="23.125" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="42.625" customWidth="1"/>
+    <col min="7" max="7" width="36.625" customWidth="1"/>
+    <col min="8" max="8" width="13.625" customWidth="1"/>
+    <col min="9" max="9" width="23.125" customWidth="1"/>
     <col min="10" max="10" width="42.125" customWidth="1"/>
     <col min="11" max="11" width="41.125" customWidth="1"/>
     <col min="12" max="12" width="35" customWidth="1"/>
-    <col min="13" max="13" width="35.125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="35.125" customWidth="1"/>
     <col min="14" max="14" width="32" customWidth="1"/>
     <col min="15" max="15" width="30.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="90.6" x14ac:dyDescent="1.2">
       <c r="A1" s="28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1"/>
       <c r="D1" s="12"/>
@@ -8674,16 +8852,16 @@
     </row>
     <row r="2" spans="1:17" ht="90.6" x14ac:dyDescent="1.2">
       <c r="A2" s="29" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M2" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="Q2" s="14"/>
     </row>
     <row r="3" spans="1:17" ht="46.05" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B3" s="30"/>
-      <c r="C3" s="95"/>
+      <c r="C3" s="77"/>
       <c r="E3" s="30"/>
       <c r="G3" s="30"/>
       <c r="H3" s="30"/>
@@ -8699,116 +8877,117 @@
       <c r="Q3" s="15"/>
     </row>
     <row r="4" spans="1:17" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="91" t="s">
+      <c r="C4" s="73" t="s">
+        <v>138</v>
+      </c>
+      <c r="D4" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="60" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="78" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="54" t="s">
+        <v>137</v>
+      </c>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="52" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" s="52" t="s">
+        <v>17</v>
+      </c>
+      <c r="M4" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="N4" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="O4" s="53" t="s">
         <v>139</v>
       </c>
-      <c r="D4" s="56" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="66" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="67" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="60" t="s">
-        <v>138</v>
-      </c>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
-      <c r="J4" s="57" t="s">
-        <v>12</v>
-      </c>
-      <c r="K4" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="L4" s="57" t="s">
-        <v>17</v>
-      </c>
-      <c r="M4" s="57" t="s">
-        <v>18</v>
-      </c>
-      <c r="N4" s="57" t="s">
-        <v>19</v>
-      </c>
-      <c r="O4" s="58" t="s">
-        <v>28</v>
-      </c>
     </row>
     <row r="5" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="44" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="87" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="92" t="str">
+      <c r="C5" s="74" t="str">
         <f ca="1">IF(E5="","",
  IF(OR(G5=1,G5=100%),"Done",
   6 - MAX(1,MIN(5,
     1+(E5-TODAY()&lt;=30)+(E5-TODAY()&lt;=14)+(E5-TODAY()&lt;=7)+(E5-TODAY()&lt;=3)
     -IF(IF(G5&gt;1,G5/100,G5)&gt;=0.8,2,IF(IF(G5&gt;1,G5/100,G5)&gt;=0.5,1,0))
   ))
- )
-)</f>
+ ))</f>
         <v>Done</v>
       </c>
-      <c r="D5" s="83">
+      <c r="D5" s="85">
         <v>45921</v>
       </c>
-      <c r="E5" s="68">
+      <c r="E5" s="61">
         <v>45934</v>
       </c>
-      <c r="F5" s="69"/>
-      <c r="G5" s="61">
+      <c r="F5" s="79"/>
+      <c r="G5" s="55">
         <v>1</v>
       </c>
-      <c r="H5" s="82">
+      <c r="H5" s="68">
         <f xml:space="preserve"> G5*100</f>
         <v>100</v>
       </c>
-      <c r="I5" s="82">
+      <c r="I5" s="68">
         <f xml:space="preserve"> 100 - H5</f>
         <v>0</v>
       </c>
-      <c r="J5" s="49">
-        <f>$J$3</f>
+      <c r="J5" s="46">
+        <f t="shared" ref="J5:J29" si="0">$J$3</f>
         <v>45921</v>
       </c>
-      <c r="K5" s="50">
-        <f>IF(ISBLANK(D5),0,D5-J5)</f>
-        <v>0</v>
-      </c>
-      <c r="L5" s="50">
-        <f>$G5*$O5</f>
-        <v>13</v>
-      </c>
-      <c r="M5" s="50">
+      <c r="K5" s="47">
+        <f t="shared" ref="K5:K29" si="1">IF(ISBLANK(D5),0,D5-J5)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="47">
+        <f t="shared" ref="L5:L29" si="2">$G5*$O5</f>
+        <v>10</v>
+      </c>
+      <c r="M5" s="47">
         <f>O5-L5</f>
         <v>0</v>
       </c>
-      <c r="N5" s="50">
-        <f>IF(ISBLANK(F5),0,(F5-D5)-O5)</f>
-        <v>0</v>
-      </c>
-      <c r="O5" s="51">
-        <f>IF(ISBLANK(E5),0,E5-D5)</f>
-        <v>13</v>
+      <c r="N5" s="94">
+        <f t="shared" ref="N5:N29" si="3">IF(ISBLANK(F5),0,(F5-D5)-O5)</f>
+        <v>0</v>
+      </c>
+      <c r="O5" s="97">
+        <f>IF(ISBLANK(E5), 0,
+   SIGN(E5-D5) * NETWORKDAYS( D5 + SIGN(E5-D5), E5, $H$2:$H$50 )
+)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="26"/>
-      <c r="B6" s="88" t="s">
-        <v>135</v>
-      </c>
-      <c r="C6" s="92">
-        <f t="shared" ref="C6:C29" ca="1" si="0">IF(E6="","",
+      <c r="B6" s="70" t="s">
+        <v>134</v>
+      </c>
+      <c r="C6" s="74">
+        <f t="shared" ref="C6:C29" ca="1" si="4">IF(E6="","",
  IF(OR(G6=1,G6=100%),"Done",
   6 - MAX(1,MIN(5,
     1+(E6-TODAY()&lt;=30)+(E6-TODAY()&lt;=14)+(E6-TODAY()&lt;=7)+(E6-TODAY()&lt;=3)
@@ -8818,1300 +8997,1288 @@
 )</f>
         <v>2</v>
       </c>
-      <c r="D6" s="84">
+      <c r="D6" s="86">
         <v>45928</v>
       </c>
-      <c r="E6" s="59">
+      <c r="E6" s="87">
         <v>45949</v>
       </c>
-      <c r="F6" s="70"/>
-      <c r="G6" s="62">
+      <c r="F6" s="80"/>
+      <c r="G6" s="56">
         <v>0.5</v>
       </c>
-      <c r="H6" s="82">
-        <f t="shared" ref="H6:H29" si="1" xml:space="preserve"> G6*100</f>
+      <c r="H6" s="68">
+        <f t="shared" ref="H6:H29" si="5" xml:space="preserve"> G6*100</f>
         <v>50</v>
       </c>
-      <c r="I6" s="82">
-        <f t="shared" ref="I6:I29" si="2" xml:space="preserve"> 100 - H6</f>
+      <c r="I6" s="68">
+        <f t="shared" ref="I6:I29" si="6" xml:space="preserve"> 100 - H6</f>
         <v>50</v>
       </c>
-      <c r="J6" s="35">
-        <f>$J$3</f>
+      <c r="J6" s="34">
+        <f t="shared" si="0"/>
         <v>45921</v>
       </c>
-      <c r="K6" s="36">
-        <f>IF(ISBLANK(D6),0,D6-J6)</f>
+      <c r="K6" s="35">
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="L6" s="36">
-        <f>$G6*$O6</f>
-        <v>10.5</v>
-      </c>
-      <c r="M6" s="36">
-        <f t="shared" ref="M6:M12" si="3">O6-L6</f>
-        <v>10.5</v>
-      </c>
-      <c r="N6" s="36">
-        <f>IF(ISBLANK(F6),0,(F6-D6)-O6)</f>
-        <v>0</v>
-      </c>
-      <c r="O6" s="37">
-        <f>IF(ISBLANK(E6),0,E6-D6)</f>
-        <v>21</v>
+      <c r="L6" s="35">
+        <f t="shared" si="2"/>
+        <v>7.5</v>
+      </c>
+      <c r="M6" s="35">
+        <f t="shared" ref="M6:M12" si="7">O6-L6</f>
+        <v>7.5</v>
+      </c>
+      <c r="N6" s="95">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O6" s="98">
+        <f t="shared" ref="O6:O29" si="8">IF(ISBLANK(E6), 0,
+   SIGN(E6-D6) * NETWORKDAYS( D6 + SIGN(E6-D6), E6, $H$2:$H$50 )
+)</f>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="26"/>
-      <c r="B7" s="88" t="s">
-        <v>136</v>
-      </c>
-      <c r="C7" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B7" s="70" t="s">
+        <v>135</v>
+      </c>
+      <c r="C7" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>1</v>
       </c>
-      <c r="D7" s="84">
+      <c r="D7" s="86">
         <v>45928</v>
       </c>
-      <c r="E7" s="59">
+      <c r="E7" s="87">
         <v>45949</v>
       </c>
-      <c r="F7" s="70"/>
-      <c r="G7" s="62">
+      <c r="F7" s="80"/>
+      <c r="G7" s="56">
         <v>0.1</v>
       </c>
-      <c r="H7" s="82">
+      <c r="H7" s="68">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="I7" s="68">
+        <f t="shared" si="6"/>
+        <v>90</v>
+      </c>
+      <c r="J7" s="34">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K7" s="35">
         <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="I7" s="82">
+        <v>7</v>
+      </c>
+      <c r="L7" s="35">
         <f t="shared" si="2"/>
-        <v>90</v>
-      </c>
-      <c r="J7" s="35">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K7" s="36">
-        <f>IF(ISBLANK(D7),0,D7-J7)</f>
-        <v>7</v>
-      </c>
-      <c r="L7" s="36">
-        <f>$G7*$O7</f>
-        <v>2.1</v>
-      </c>
-      <c r="M7" s="36">
-        <f t="shared" ref="M7" si="4">O7-L7</f>
-        <v>18.899999999999999</v>
-      </c>
-      <c r="N7" s="36">
-        <f>IF(ISBLANK(F7),0,(F7-D7)-O7)</f>
-        <v>0</v>
-      </c>
-      <c r="O7" s="37">
-        <f>IF(ISBLANK(E7),0,E7-D7)</f>
-        <v>21</v>
+        <v>1.5</v>
+      </c>
+      <c r="M7" s="35">
+        <f t="shared" ref="M7" si="9">O7-L7</f>
+        <v>13.5</v>
+      </c>
+      <c r="N7" s="95">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O7" s="98">
+        <f t="shared" si="8"/>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="26"/>
-      <c r="B8" s="89" t="s">
-        <v>50</v>
-      </c>
-      <c r="C8" s="92" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B8" s="71" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="74" t="str">
+        <f t="shared" ca="1" si="4"/>
         <v>Done</v>
       </c>
-      <c r="D8" s="85">
+      <c r="D8" s="88">
         <v>45944</v>
       </c>
-      <c r="E8" s="71">
+      <c r="E8" s="65">
         <v>45954</v>
       </c>
-      <c r="F8" s="72"/>
-      <c r="G8" s="63">
+      <c r="F8" s="81"/>
+      <c r="G8" s="57">
         <v>1</v>
       </c>
-      <c r="H8" s="82">
+      <c r="H8" s="68">
+        <f t="shared" si="5"/>
+        <v>100</v>
+      </c>
+      <c r="I8" s="68">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J8" s="48">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K8" s="49">
         <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+      <c r="L8" s="49">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="M8" s="49">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="N8" s="96">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O8" s="99">
+        <f t="shared" si="8"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="69" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="74" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Done</v>
+      </c>
+      <c r="D9" s="85">
+        <v>45940</v>
+      </c>
+      <c r="E9" s="61">
+        <v>45960</v>
+      </c>
+      <c r="F9" s="82"/>
+      <c r="G9" s="58">
+        <v>1</v>
+      </c>
+      <c r="H9" s="68">
+        <f t="shared" si="5"/>
         <v>100</v>
       </c>
-      <c r="I8" s="82">
+      <c r="I9" s="68">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J9" s="32">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K9" s="33">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="L9" s="33">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J8" s="52">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K8" s="53">
-        <f>IF(ISBLANK(D8),0,D8-J8)</f>
-        <v>23</v>
-      </c>
-      <c r="L8" s="53">
-        <f>$G8*$O8</f>
-        <v>10</v>
-      </c>
-      <c r="M8" s="53">
+        <v>14</v>
+      </c>
+      <c r="M9" s="33">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="N9" s="100">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="N8" s="53">
-        <f>IF(ISBLANK(F8),0,(F8-D8)-O8)</f>
-        <v>0</v>
-      </c>
-      <c r="O8" s="54">
-        <f>IF(ISBLANK(E8),0,E8-D8)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="47" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="87" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="92" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>Done</v>
-      </c>
-      <c r="D9" s="83">
-        <v>45940</v>
-      </c>
-      <c r="E9" s="68">
-        <v>45960</v>
-      </c>
-      <c r="F9" s="73"/>
-      <c r="G9" s="64">
-        <v>1</v>
-      </c>
-      <c r="H9" s="82">
-        <f t="shared" si="1"/>
-        <v>100</v>
-      </c>
-      <c r="I9" s="82">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J9" s="32">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K9" s="33">
-        <f>IF(ISBLANK(D9),0,D9-J9)</f>
-        <v>19</v>
-      </c>
-      <c r="L9" s="33">
-        <f>$G9*$O9</f>
-        <v>20</v>
-      </c>
-      <c r="M9" s="33">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="N9" s="33">
-        <f>IF(ISBLANK(F9),0,(F9-D9)-O9)</f>
-        <v>0</v>
-      </c>
-      <c r="O9" s="34">
-        <f>IF(ISBLANK(E9),0,E9-D9)</f>
-        <v>20</v>
+      <c r="O9" s="97">
+        <f t="shared" si="8"/>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26"/>
-      <c r="B10" s="88" t="s">
-        <v>132</v>
-      </c>
-      <c r="C10" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B10" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>4</v>
       </c>
-      <c r="D10" s="84">
+      <c r="D10" s="86">
         <v>45959</v>
       </c>
-      <c r="E10" s="59">
+      <c r="E10" s="87">
         <v>45970</v>
       </c>
-      <c r="F10" s="70"/>
-      <c r="G10" s="62">
-        <v>0</v>
-      </c>
-      <c r="H10" s="82">
+      <c r="F10" s="80"/>
+      <c r="G10" s="56">
+        <v>0</v>
+      </c>
+      <c r="H10" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I10" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J10" s="34">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K10" s="35">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I10" s="82">
+        <v>38</v>
+      </c>
+      <c r="L10" s="35">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J10" s="35">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K10" s="36">
-        <f>IF(ISBLANK(D10),0,D10-J10)</f>
-        <v>38</v>
-      </c>
-      <c r="L10" s="36">
-        <f>$G10*$O10</f>
-        <v>0</v>
-      </c>
-      <c r="M10" s="36">
+        <v>0</v>
+      </c>
+      <c r="M10" s="35">
+        <f t="shared" si="7"/>
+        <v>7</v>
+      </c>
+      <c r="N10" s="95">
         <f t="shared" si="3"/>
-        <v>11</v>
-      </c>
-      <c r="N10" s="36">
-        <f>IF(ISBLANK(F10),0,(F10-D10)-O10)</f>
-        <v>0</v>
-      </c>
-      <c r="O10" s="37">
-        <f>IF(ISBLANK(E10),0,E10-D10)</f>
-        <v>11</v>
+        <v>0</v>
+      </c>
+      <c r="O10" s="98">
+        <f t="shared" si="8"/>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="26"/>
-      <c r="B11" s="88" t="s">
-        <v>133</v>
-      </c>
-      <c r="C11" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B11" s="70" t="s">
+        <v>132</v>
+      </c>
+      <c r="C11" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>4</v>
       </c>
-      <c r="D11" s="84">
+      <c r="D11" s="86">
         <v>45970</v>
       </c>
-      <c r="E11" s="59">
+      <c r="E11" s="87">
         <v>45977</v>
       </c>
-      <c r="F11" s="70"/>
-      <c r="G11" s="62">
-        <v>0</v>
-      </c>
-      <c r="H11" s="82">
+      <c r="F11" s="80"/>
+      <c r="G11" s="56">
+        <v>0</v>
+      </c>
+      <c r="H11" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I11" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J11" s="34">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K11" s="35">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I11" s="82">
+        <v>49</v>
+      </c>
+      <c r="L11" s="35">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J11" s="35">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K11" s="36">
-        <f>IF(ISBLANK(D11),0,D11-J11)</f>
-        <v>49</v>
-      </c>
-      <c r="L11" s="36">
-        <f>$G11*$O11</f>
-        <v>0</v>
-      </c>
-      <c r="M11" s="36">
+        <v>0</v>
+      </c>
+      <c r="M11" s="35">
+        <f t="shared" si="7"/>
+        <v>5</v>
+      </c>
+      <c r="N11" s="95">
         <f t="shared" si="3"/>
-        <v>7</v>
-      </c>
-      <c r="N11" s="36">
-        <f>IF(ISBLANK(F11),0,(F11-D11)-O11)</f>
-        <v>0</v>
-      </c>
-      <c r="O11" s="37">
-        <f>IF(ISBLANK(E11),0,E11-D11)</f>
-        <v>7</v>
+        <v>0</v>
+      </c>
+      <c r="O11" s="98">
+        <f t="shared" si="8"/>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="27"/>
-      <c r="B12" s="90" t="s">
-        <v>134</v>
-      </c>
-      <c r="C12" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B12" s="72" t="s">
+        <v>133</v>
+      </c>
+      <c r="C12" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D12" s="84">
+      <c r="D12" s="89">
         <v>45977</v>
       </c>
-      <c r="E12" s="71">
-        <v>46021</v>
-      </c>
-      <c r="F12" s="72"/>
-      <c r="G12" s="65">
-        <v>0</v>
-      </c>
-      <c r="H12" s="82">
+      <c r="E12" s="90">
+        <v>45984</v>
+      </c>
+      <c r="F12" s="81"/>
+      <c r="G12" s="59">
+        <v>0</v>
+      </c>
+      <c r="H12" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I12" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J12" s="36">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K12" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I12" s="82">
+        <v>56</v>
+      </c>
+      <c r="L12" s="37">
         <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M12" s="37">
+        <f t="shared" si="7"/>
+        <v>5</v>
+      </c>
+      <c r="N12" s="101">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O12" s="99">
+        <f t="shared" si="8"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="69" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="91">
+        <f t="shared" ca="1" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="D13" s="85">
+        <v>45981</v>
+      </c>
+      <c r="E13" s="61">
+        <v>45988</v>
+      </c>
+      <c r="F13" s="82"/>
+      <c r="G13" s="58">
+        <v>0</v>
+      </c>
+      <c r="H13" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I13" s="68">
+        <f t="shared" si="6"/>
         <v>100</v>
       </c>
-      <c r="J12" s="38">
-        <f>$J$3</f>
+      <c r="J13" s="32">
+        <f t="shared" si="0"/>
         <v>45921</v>
       </c>
-      <c r="K12" s="39">
-        <f>IF(ISBLANK(D12),0,D12-J12)</f>
-        <v>56</v>
-      </c>
-      <c r="L12" s="39">
-        <f>$G12*$O12</f>
-        <v>0</v>
-      </c>
-      <c r="M12" s="39">
+      <c r="K13" s="33">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+      <c r="L13" s="33">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M13" s="33">
+        <f t="shared" ref="M13:M27" si="10">O13-L13</f>
+        <v>5</v>
+      </c>
+      <c r="N13" s="100">
         <f t="shared" si="3"/>
-        <v>44</v>
-      </c>
-      <c r="N12" s="39">
-        <f>IF(ISBLANK(F12),0,(F12-D12)-O12)</f>
-        <v>0</v>
-      </c>
-      <c r="O12" s="40">
-        <f>IF(ISBLANK(E12),0,E12-D12)</f>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="B13" s="87" t="s">
-        <v>70</v>
-      </c>
-      <c r="C13" s="92">
-        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O13" s="97">
+        <f t="shared" si="8"/>
         <v>5</v>
-      </c>
-      <c r="D13" s="83">
-        <v>46011</v>
-      </c>
-      <c r="E13" s="68">
-        <v>46020</v>
-      </c>
-      <c r="F13" s="73"/>
-      <c r="G13" s="64">
-        <v>0</v>
-      </c>
-      <c r="H13" s="82">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I13" s="82">
-        <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J13" s="32">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K13" s="33">
-        <f>IF(ISBLANK(D13),0,D13-J13)</f>
-        <v>90</v>
-      </c>
-      <c r="L13" s="33">
-        <f>$G13*$O13</f>
-        <v>0</v>
-      </c>
-      <c r="M13" s="33">
-        <f t="shared" ref="M13:M27" si="5">O13-L13</f>
-        <v>9</v>
-      </c>
-      <c r="N13" s="33">
-        <f>IF(ISBLANK(F13),0,(F13-D13)-O13)</f>
-        <v>0</v>
-      </c>
-      <c r="O13" s="34">
-        <f>IF(ISBLANK(E13),0,E13-D13)</f>
-        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="26"/>
-      <c r="B14" s="88" t="s">
-        <v>74</v>
-      </c>
-      <c r="C14" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B14" s="70" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="91">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D14" s="84">
-        <v>46020</v>
-      </c>
-      <c r="E14" s="59">
-        <v>46030</v>
-      </c>
-      <c r="F14" s="70"/>
-      <c r="G14" s="62">
-        <v>0</v>
-      </c>
-      <c r="H14" s="82">
+      <c r="D14" s="86">
+        <v>45988</v>
+      </c>
+      <c r="E14" s="87">
+        <v>45999</v>
+      </c>
+      <c r="F14" s="80"/>
+      <c r="G14" s="56">
+        <v>0</v>
+      </c>
+      <c r="H14" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I14" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J14" s="34">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K14" s="35">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I14" s="82">
+        <v>67</v>
+      </c>
+      <c r="L14" s="35">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J14" s="35">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K14" s="36">
-        <f>IF(ISBLANK(D14),0,D14-J14)</f>
-        <v>99</v>
-      </c>
-      <c r="L14" s="36">
-        <f>$G14*$O14</f>
-        <v>0</v>
-      </c>
-      <c r="M14" s="36">
-        <f t="shared" si="5"/>
-        <v>10</v>
-      </c>
-      <c r="N14" s="36">
-        <f>IF(ISBLANK(F14),0,(F14-D14)-O14)</f>
-        <v>0</v>
-      </c>
-      <c r="O14" s="37">
-        <f>IF(ISBLANK(E14),0,E14-D14)</f>
-        <v>10</v>
+        <v>0</v>
+      </c>
+      <c r="M14" s="35">
+        <f t="shared" si="10"/>
+        <v>7</v>
+      </c>
+      <c r="N14" s="95">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O14" s="98">
+        <f t="shared" si="8"/>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="27"/>
-      <c r="B15" s="90" t="s">
-        <v>77</v>
-      </c>
-      <c r="C15" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B15" s="72" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="91">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D15" s="85">
-        <v>46025</v>
-      </c>
-      <c r="E15" s="71">
+      <c r="D15" s="88">
+        <v>45994</v>
+      </c>
+      <c r="E15" s="65">
         <v>46046</v>
       </c>
-      <c r="F15" s="72"/>
-      <c r="G15" s="65">
-        <v>0</v>
-      </c>
-      <c r="H15" s="82">
+      <c r="F15" s="81"/>
+      <c r="G15" s="59">
+        <v>0</v>
+      </c>
+      <c r="H15" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I15" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J15" s="36">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K15" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I15" s="82">
+        <v>73</v>
+      </c>
+      <c r="L15" s="37">
         <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M15" s="37">
+        <f t="shared" si="10"/>
+        <v>37</v>
+      </c>
+      <c r="N15" s="101">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O15" s="102">
+        <f t="shared" si="8"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="44" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" s="69" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16" s="74">
+        <f t="shared" ca="1" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="D16" s="92">
+        <v>46046</v>
+      </c>
+      <c r="E16" s="93">
+        <v>46061</v>
+      </c>
+      <c r="F16" s="82"/>
+      <c r="G16" s="58">
+        <v>0</v>
+      </c>
+      <c r="H16" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I16" s="68">
+        <f t="shared" si="6"/>
         <v>100</v>
       </c>
-      <c r="J15" s="38">
-        <f>$J$3</f>
+      <c r="J16" s="32">
+        <f t="shared" si="0"/>
         <v>45921</v>
       </c>
-      <c r="K15" s="39">
-        <f>IF(ISBLANK(D15),0,D15-J15)</f>
-        <v>104</v>
-      </c>
-      <c r="L15" s="39">
-        <f>$G15*$O15</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="39">
-        <f t="shared" si="5"/>
-        <v>21</v>
-      </c>
-      <c r="N15" s="39">
-        <f>IF(ISBLANK(F15),0,(F15-D15)-O15)</f>
-        <v>0</v>
-      </c>
-      <c r="O15" s="40">
-        <f>IF(ISBLANK(E15),0,E15-D15)</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="47" t="s">
-        <v>81</v>
-      </c>
-      <c r="B16" s="87" t="s">
-        <v>82</v>
-      </c>
-      <c r="C16" s="92">
-        <f t="shared" ca="1" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="D16" s="83">
-        <v>46046</v>
-      </c>
-      <c r="E16" s="68">
-        <v>46061</v>
-      </c>
-      <c r="F16" s="73"/>
-      <c r="G16" s="64">
-        <v>0</v>
-      </c>
-      <c r="H16" s="82">
+      <c r="K16" s="33">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I16" s="82">
+        <v>125</v>
+      </c>
+      <c r="L16" s="33">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J16" s="32">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K16" s="33">
-        <f>IF(ISBLANK(D16),0,D16-J16)</f>
-        <v>125</v>
-      </c>
-      <c r="L16" s="33">
-        <f>$G16*$O16</f>
         <v>0</v>
       </c>
       <c r="M16" s="33">
-        <f t="shared" si="5"/>
-        <v>15</v>
-      </c>
-      <c r="N16" s="33">
-        <f>IF(ISBLANK(F16),0,(F16-D16)-O16)</f>
-        <v>0</v>
-      </c>
-      <c r="O16" s="34">
-        <f>IF(ISBLANK(E16),0,E16-D16)</f>
-        <v>15</v>
+        <f t="shared" si="10"/>
+        <v>10</v>
+      </c>
+      <c r="N16" s="100">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O16" s="97">
+        <f t="shared" si="8"/>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26"/>
-      <c r="B17" s="88" t="s">
-        <v>85</v>
-      </c>
-      <c r="C17" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B17" s="70" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D17" s="84">
+      <c r="D17" s="86">
         <v>46061</v>
       </c>
-      <c r="E17" s="59">
+      <c r="E17" s="87">
         <v>46077</v>
       </c>
-      <c r="F17" s="70"/>
-      <c r="G17" s="62">
-        <v>0</v>
-      </c>
-      <c r="H17" s="82">
+      <c r="F17" s="80"/>
+      <c r="G17" s="56">
+        <v>0</v>
+      </c>
+      <c r="H17" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I17" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J17" s="34">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K17" s="35">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I17" s="82">
+        <v>140</v>
+      </c>
+      <c r="L17" s="35">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J17" s="35">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K17" s="36">
-        <f>IF(ISBLANK(D17),0,D17-J17)</f>
-        <v>140</v>
-      </c>
-      <c r="L17" s="36">
-        <f>$G17*$O17</f>
-        <v>0</v>
-      </c>
-      <c r="M17" s="36">
-        <f t="shared" si="5"/>
-        <v>16</v>
-      </c>
-      <c r="N17" s="36">
-        <f>IF(ISBLANK(F17),0,(F17-D17)-O17)</f>
-        <v>0</v>
-      </c>
-      <c r="O17" s="37">
-        <f>IF(ISBLANK(E17),0,E17-D17)</f>
-        <v>16</v>
+        <v>0</v>
+      </c>
+      <c r="M17" s="35">
+        <f t="shared" si="10"/>
+        <v>12</v>
+      </c>
+      <c r="N17" s="95">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O17" s="98">
+        <f t="shared" si="8"/>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26"/>
-      <c r="B18" s="88" t="s">
-        <v>88</v>
-      </c>
-      <c r="C18" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B18" s="70" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D18" s="84">
+      <c r="D18" s="86">
         <v>46077</v>
       </c>
-      <c r="E18" s="59">
+      <c r="E18" s="87">
         <v>46097</v>
       </c>
-      <c r="F18" s="70"/>
-      <c r="G18" s="62">
-        <v>0</v>
-      </c>
-      <c r="H18" s="82">
+      <c r="F18" s="80"/>
+      <c r="G18" s="56">
+        <v>0</v>
+      </c>
+      <c r="H18" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I18" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J18" s="34">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K18" s="35">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I18" s="82">
+        <v>156</v>
+      </c>
+      <c r="L18" s="35">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J18" s="35">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K18" s="36">
-        <f>IF(ISBLANK(D18),0,D18-J18)</f>
-        <v>156</v>
-      </c>
-      <c r="L18" s="36">
-        <f>$G18*$O18</f>
-        <v>0</v>
-      </c>
-      <c r="M18" s="36">
-        <f t="shared" si="5"/>
-        <v>20</v>
-      </c>
-      <c r="N18" s="36">
-        <f>IF(ISBLANK(F18),0,(F18-D18)-O18)</f>
-        <v>0</v>
-      </c>
-      <c r="O18" s="37">
-        <f>IF(ISBLANK(E18),0,E18-D18)</f>
-        <v>20</v>
+        <v>0</v>
+      </c>
+      <c r="M18" s="35">
+        <f t="shared" si="10"/>
+        <v>14</v>
+      </c>
+      <c r="N18" s="95">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O18" s="98">
+        <f t="shared" si="8"/>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="27"/>
-      <c r="B19" s="90" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B19" s="72" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D19" s="85">
+      <c r="D19" s="88">
         <v>46092</v>
       </c>
-      <c r="E19" s="71">
+      <c r="E19" s="65">
         <v>46101</v>
       </c>
-      <c r="F19" s="72"/>
-      <c r="G19" s="65">
-        <v>0</v>
-      </c>
-      <c r="H19" s="82">
+      <c r="F19" s="81"/>
+      <c r="G19" s="59">
+        <v>0</v>
+      </c>
+      <c r="H19" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I19" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J19" s="36">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K19" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I19" s="82">
+        <v>171</v>
+      </c>
+      <c r="L19" s="37">
         <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M19" s="37">
+        <f t="shared" si="10"/>
+        <v>7</v>
+      </c>
+      <c r="N19" s="101">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O19" s="99">
+        <f t="shared" si="8"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="C20" s="74">
+        <f t="shared" ca="1" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="D20" s="85">
+        <v>46101</v>
+      </c>
+      <c r="E20" s="61">
+        <v>46105</v>
+      </c>
+      <c r="F20" s="82"/>
+      <c r="G20" s="58">
+        <v>0</v>
+      </c>
+      <c r="H20" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I20" s="68">
+        <f t="shared" si="6"/>
         <v>100</v>
       </c>
-      <c r="J19" s="38">
-        <f>$J$3</f>
+      <c r="J20" s="32">
+        <f t="shared" si="0"/>
         <v>45921</v>
       </c>
-      <c r="K19" s="39">
-        <f>IF(ISBLANK(D19),0,D19-J19)</f>
-        <v>171</v>
-      </c>
-      <c r="L19" s="39">
-        <f>$G19*$O19</f>
-        <v>0</v>
-      </c>
-      <c r="M19" s="39">
-        <f t="shared" si="5"/>
-        <v>9</v>
-      </c>
-      <c r="N19" s="39">
-        <f>IF(ISBLANK(F19),0,(F19-D19)-O19)</f>
-        <v>0</v>
-      </c>
-      <c r="O19" s="40">
-        <f>IF(ISBLANK(E19),0,E19-D19)</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="47" t="s">
-        <v>95</v>
-      </c>
-      <c r="B20" s="87" t="s">
-        <v>96</v>
-      </c>
-      <c r="C20" s="92">
-        <f t="shared" ca="1" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="D20" s="83">
-        <v>46101</v>
-      </c>
-      <c r="E20" s="68">
-        <v>46105</v>
-      </c>
-      <c r="F20" s="73"/>
-      <c r="G20" s="64">
-        <v>0</v>
-      </c>
-      <c r="H20" s="82">
+      <c r="K20" s="33">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I20" s="82">
+        <v>180</v>
+      </c>
+      <c r="L20" s="33">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J20" s="32">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K20" s="33">
-        <f>IF(ISBLANK(D20),0,D20-J20)</f>
-        <v>180</v>
-      </c>
-      <c r="L20" s="33">
-        <f>$G20*$O20</f>
         <v>0</v>
       </c>
       <c r="M20" s="33">
-        <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="N20" s="33">
-        <f>IF(ISBLANK(F20),0,(F20-D20)-O20)</f>
-        <v>0</v>
-      </c>
-      <c r="O20" s="34">
-        <f>IF(ISBLANK(E20),0,E20-D20)</f>
-        <v>4</v>
+        <f t="shared" si="10"/>
+        <v>2</v>
+      </c>
+      <c r="N20" s="100">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O20" s="97">
+        <f t="shared" si="8"/>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="26"/>
-      <c r="B21" s="88" t="s">
+      <c r="B21" s="70" t="s">
+        <v>99</v>
+      </c>
+      <c r="C21" s="74">
+        <f t="shared" ca="1" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="D21" s="86">
+        <v>46105</v>
+      </c>
+      <c r="E21" s="87">
+        <v>46125</v>
+      </c>
+      <c r="F21" s="80"/>
+      <c r="G21" s="56">
+        <v>0</v>
+      </c>
+      <c r="H21" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I21" s="68">
+        <f t="shared" si="6"/>
         <v>100</v>
       </c>
-      <c r="C21" s="92">
-        <f t="shared" ca="1" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="D21" s="84">
-        <v>46105</v>
-      </c>
-      <c r="E21" s="59">
-        <v>46125</v>
-      </c>
-      <c r="F21" s="70"/>
-      <c r="G21" s="62">
-        <v>0</v>
-      </c>
-      <c r="H21" s="82">
+      <c r="J21" s="34">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K21" s="35">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I21" s="82">
+        <v>184</v>
+      </c>
+      <c r="L21" s="35">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J21" s="35">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K21" s="36">
-        <f>IF(ISBLANK(D21),0,D21-J21)</f>
-        <v>184</v>
-      </c>
-      <c r="L21" s="36">
-        <f>$G21*$O21</f>
-        <v>0</v>
-      </c>
-      <c r="M21" s="36">
-        <f t="shared" si="5"/>
-        <v>20</v>
-      </c>
-      <c r="N21" s="36">
-        <f>IF(ISBLANK(F21),0,(F21-D21)-O21)</f>
-        <v>0</v>
-      </c>
-      <c r="O21" s="37">
-        <f>IF(ISBLANK(E21),0,E21-D21)</f>
-        <v>20</v>
+        <v>0</v>
+      </c>
+      <c r="M21" s="35">
+        <f t="shared" si="10"/>
+        <v>14</v>
+      </c>
+      <c r="N21" s="95">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O21" s="98">
+        <f t="shared" si="8"/>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="27"/>
-      <c r="B22" s="90" t="s">
-        <v>104</v>
-      </c>
-      <c r="C22" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B22" s="72" t="s">
+        <v>103</v>
+      </c>
+      <c r="C22" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D22" s="85">
+      <c r="D22" s="88">
         <v>46110</v>
       </c>
-      <c r="E22" s="71">
+      <c r="E22" s="65">
         <v>46130</v>
       </c>
-      <c r="F22" s="72"/>
-      <c r="G22" s="65">
-        <v>0</v>
-      </c>
-      <c r="H22" s="82">
+      <c r="F22" s="81"/>
+      <c r="G22" s="59">
+        <v>0</v>
+      </c>
+      <c r="H22" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I22" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J22" s="36">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K22" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I22" s="82">
+        <v>189</v>
+      </c>
+      <c r="L22" s="37">
         <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M22" s="37">
+        <f t="shared" si="10"/>
+        <v>15</v>
+      </c>
+      <c r="N22" s="101">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O22" s="99">
+        <f t="shared" si="8"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="44" t="s">
+        <v>106</v>
+      </c>
+      <c r="B23" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="C23" s="74">
+        <f t="shared" ca="1" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="D23" s="85">
+        <v>46125</v>
+      </c>
+      <c r="E23" s="61">
+        <v>46136</v>
+      </c>
+      <c r="F23" s="82"/>
+      <c r="G23" s="58">
+        <v>0</v>
+      </c>
+      <c r="H23" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I23" s="68">
+        <f t="shared" si="6"/>
         <v>100</v>
       </c>
-      <c r="J22" s="38">
-        <f>$J$3</f>
+      <c r="J23" s="32">
+        <f t="shared" si="0"/>
         <v>45921</v>
       </c>
-      <c r="K22" s="39">
-        <f>IF(ISBLANK(D22),0,D22-J22)</f>
-        <v>189</v>
-      </c>
-      <c r="L22" s="39">
-        <f>$G22*$O22</f>
-        <v>0</v>
-      </c>
-      <c r="M22" s="39">
-        <f t="shared" si="5"/>
-        <v>20</v>
-      </c>
-      <c r="N22" s="39">
-        <f>IF(ISBLANK(F22),0,(F22-D22)-O22)</f>
-        <v>0</v>
-      </c>
-      <c r="O22" s="40">
-        <f>IF(ISBLANK(E22),0,E22-D22)</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="47" t="s">
-        <v>107</v>
-      </c>
-      <c r="B23" s="87" t="s">
-        <v>108</v>
-      </c>
-      <c r="C23" s="92">
-        <f t="shared" ca="1" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="D23" s="83">
-        <v>46125</v>
-      </c>
-      <c r="E23" s="68">
-        <v>46136</v>
-      </c>
-      <c r="F23" s="73"/>
-      <c r="G23" s="64">
-        <v>0</v>
-      </c>
-      <c r="H23" s="82">
+      <c r="K23" s="33">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I23" s="82">
+        <v>204</v>
+      </c>
+      <c r="L23" s="33">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J23" s="32">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K23" s="33">
-        <f>IF(ISBLANK(D23),0,D23-J23)</f>
-        <v>204</v>
-      </c>
-      <c r="L23" s="33">
-        <f>$G23*$O23</f>
         <v>0</v>
       </c>
       <c r="M23" s="33">
-        <f t="shared" si="5"/>
-        <v>11</v>
-      </c>
-      <c r="N23" s="33">
-        <f>IF(ISBLANK(F23),0,(F23-D23)-O23)</f>
-        <v>0</v>
-      </c>
-      <c r="O23" s="34">
-        <f>IF(ISBLANK(E23),0,E23-D23)</f>
-        <v>11</v>
+        <f t="shared" si="10"/>
+        <v>9</v>
+      </c>
+      <c r="N23" s="100">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O23" s="97">
+        <f t="shared" si="8"/>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="27"/>
-      <c r="B24" s="90" t="s">
-        <v>111</v>
-      </c>
-      <c r="C24" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B24" s="72" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D24" s="85">
+      <c r="D24" s="88">
         <v>46132</v>
       </c>
-      <c r="E24" s="71">
+      <c r="E24" s="65">
         <v>46141</v>
       </c>
-      <c r="F24" s="72"/>
-      <c r="G24" s="65">
-        <v>0</v>
-      </c>
-      <c r="H24" s="82">
+      <c r="F24" s="81"/>
+      <c r="G24" s="59">
+        <v>0</v>
+      </c>
+      <c r="H24" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I24" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J24" s="36">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K24" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I24" s="82">
+        <v>211</v>
+      </c>
+      <c r="L24" s="37">
         <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M24" s="37">
+        <f t="shared" si="10"/>
+        <v>7</v>
+      </c>
+      <c r="N24" s="101">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O24" s="99">
+        <f t="shared" si="8"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="44" t="s">
+        <v>114</v>
+      </c>
+      <c r="B25" s="69" t="s">
+        <v>115</v>
+      </c>
+      <c r="C25" s="74">
+        <f t="shared" ca="1" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="D25" s="85">
+        <v>46115</v>
+      </c>
+      <c r="E25" s="61">
+        <v>46141</v>
+      </c>
+      <c r="F25" s="82"/>
+      <c r="G25" s="58">
+        <v>0</v>
+      </c>
+      <c r="H25" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I25" s="68">
+        <f t="shared" si="6"/>
         <v>100</v>
       </c>
-      <c r="J24" s="38">
-        <f>$J$3</f>
+      <c r="J25" s="32">
+        <f t="shared" si="0"/>
         <v>45921</v>
       </c>
-      <c r="K24" s="39">
-        <f>IF(ISBLANK(D24),0,D24-J24)</f>
-        <v>211</v>
-      </c>
-      <c r="L24" s="39">
-        <f>$G24*$O24</f>
-        <v>0</v>
-      </c>
-      <c r="M24" s="39">
-        <f t="shared" si="5"/>
-        <v>9</v>
-      </c>
-      <c r="N24" s="39">
-        <f>IF(ISBLANK(F24),0,(F24-D24)-O24)</f>
-        <v>0</v>
-      </c>
-      <c r="O24" s="40">
-        <f>IF(ISBLANK(E24),0,E24-D24)</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="47" t="s">
-        <v>115</v>
-      </c>
-      <c r="B25" s="87" t="s">
-        <v>116</v>
-      </c>
-      <c r="C25" s="92">
-        <f t="shared" ca="1" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="D25" s="83">
-        <v>46115</v>
-      </c>
-      <c r="E25" s="68">
-        <v>46141</v>
-      </c>
-      <c r="F25" s="73"/>
-      <c r="G25" s="64">
-        <v>0</v>
-      </c>
-      <c r="H25" s="82">
+      <c r="K25" s="33">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I25" s="82">
+        <v>194</v>
+      </c>
+      <c r="L25" s="33">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J25" s="32">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K25" s="33">
-        <f>IF(ISBLANK(D25),0,D25-J25)</f>
-        <v>194</v>
-      </c>
-      <c r="L25" s="33">
-        <f>$G25*$O25</f>
         <v>0</v>
       </c>
       <c r="M25" s="33">
-        <f t="shared" si="5"/>
-        <v>26</v>
-      </c>
-      <c r="N25" s="33">
-        <f>IF(ISBLANK(F25),0,(F25-D25)-O25)</f>
-        <v>0</v>
-      </c>
-      <c r="O25" s="34">
-        <f>IF(ISBLANK(E25),0,E25-D25)</f>
-        <v>26</v>
+        <f t="shared" si="10"/>
+        <v>18</v>
+      </c>
+      <c r="N25" s="100">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O25" s="97">
+        <f t="shared" si="8"/>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="26"/>
-      <c r="B26" s="88" t="s">
-        <v>119</v>
-      </c>
-      <c r="C26" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B26" s="70" t="s">
+        <v>118</v>
+      </c>
+      <c r="C26" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D26" s="84">
+      <c r="D26" s="86">
         <v>46125</v>
       </c>
-      <c r="E26" s="59">
+      <c r="E26" s="87">
         <v>46146</v>
       </c>
-      <c r="F26" s="70"/>
-      <c r="G26" s="62">
-        <v>0</v>
-      </c>
-      <c r="H26" s="82">
+      <c r="F26" s="80"/>
+      <c r="G26" s="56">
+        <v>0</v>
+      </c>
+      <c r="H26" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I26" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J26" s="34">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K26" s="35">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I26" s="82">
+        <v>204</v>
+      </c>
+      <c r="L26" s="35">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J26" s="35">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K26" s="36">
-        <f>IF(ISBLANK(D26),0,D26-J26)</f>
-        <v>204</v>
-      </c>
-      <c r="L26" s="36">
-        <f>$G26*$O26</f>
-        <v>0</v>
-      </c>
-      <c r="M26" s="36">
-        <f t="shared" si="5"/>
-        <v>21</v>
-      </c>
-      <c r="N26" s="36">
-        <f>IF(ISBLANK(F26),0,(F26-D26)-O26)</f>
-        <v>0</v>
-      </c>
-      <c r="O26" s="37">
-        <f>IF(ISBLANK(E26),0,E26-D26)</f>
-        <v>21</v>
+        <v>0</v>
+      </c>
+      <c r="M26" s="35">
+        <f t="shared" si="10"/>
+        <v>15</v>
+      </c>
+      <c r="N26" s="95">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O26" s="98">
+        <f t="shared" si="8"/>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="26"/>
-      <c r="B27" s="89" t="s">
-        <v>122</v>
-      </c>
-      <c r="C27" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="B27" s="71" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D27" s="86">
+      <c r="D27" s="89">
         <v>46141</v>
       </c>
-      <c r="E27" s="75">
+      <c r="E27" s="90">
         <v>46161</v>
       </c>
-      <c r="F27" s="76"/>
-      <c r="G27" s="63">
-        <v>0</v>
-      </c>
-      <c r="H27" s="82">
+      <c r="F27" s="83"/>
+      <c r="G27" s="57">
+        <v>0</v>
+      </c>
+      <c r="H27" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I27" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J27" s="48">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K27" s="49">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I27" s="82">
+        <v>220</v>
+      </c>
+      <c r="L27" s="49">
         <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M27" s="49">
+        <f t="shared" si="10"/>
+        <v>14</v>
+      </c>
+      <c r="N27" s="96">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O27" s="99">
+        <f t="shared" si="8"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="B28" s="75" t="s">
+        <v>129</v>
+      </c>
+      <c r="C28" s="74">
+        <f t="shared" ca="1" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="D28" s="85">
+        <v>45959</v>
+      </c>
+      <c r="E28" s="61">
+        <v>45960</v>
+      </c>
+      <c r="F28" s="79">
+        <v>45960</v>
+      </c>
+      <c r="G28" s="63">
+        <v>0</v>
+      </c>
+      <c r="H28" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I28" s="68">
+        <f t="shared" si="6"/>
         <v>100</v>
       </c>
-      <c r="J27" s="52">
-        <f>$J$3</f>
+      <c r="J28" s="32">
+        <f t="shared" si="0"/>
         <v>45921</v>
       </c>
-      <c r="K27" s="53">
-        <f>IF(ISBLANK(D27),0,D27-J27)</f>
-        <v>220</v>
-      </c>
-      <c r="L27" s="53">
-        <f>$G27*$O27</f>
-        <v>0</v>
-      </c>
-      <c r="M27" s="53">
-        <f t="shared" si="5"/>
-        <v>20</v>
-      </c>
-      <c r="N27" s="53">
-        <f>IF(ISBLANK(F27),0,(F27-D27)-O27)</f>
-        <v>0</v>
-      </c>
-      <c r="O27" s="54">
-        <f>IF(ISBLANK(E27),0,E27-D27)</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="47" t="s">
-        <v>131</v>
-      </c>
-      <c r="B28" s="93" t="s">
-        <v>130</v>
-      </c>
-      <c r="C28" s="92">
-        <f t="shared" ca="1" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="D28" s="83">
-        <v>45959</v>
-      </c>
-      <c r="E28" s="68">
-        <v>45960</v>
-      </c>
-      <c r="F28" s="69">
-        <v>45960</v>
-      </c>
-      <c r="G28" s="77">
-        <v>0</v>
-      </c>
-      <c r="H28" s="82">
+      <c r="K28" s="33">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I28" s="82">
+        <v>38</v>
+      </c>
+      <c r="L28" s="33">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J28" s="32">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K28" s="33">
-        <f>IF(ISBLANK(D28),0,D28-J28)</f>
-        <v>38</v>
-      </c>
-      <c r="L28" s="33">
-        <f>$G28*$O28</f>
         <v>0</v>
       </c>
       <c r="M28" s="33">
         <f>O28-L28</f>
         <v>1</v>
       </c>
-      <c r="N28" s="33">
-        <f>IF(ISBLANK(F28),0,(F28-D28)-O28)</f>
-        <v>0</v>
-      </c>
-      <c r="O28" s="34">
-        <f>IF(ISBLANK(E28),0,E28-D28)</f>
+      <c r="N28" s="100">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O28" s="97">
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:15" s="11" customFormat="1" ht="106.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="80"/>
-      <c r="B29" s="94" t="s">
-        <v>137</v>
-      </c>
-      <c r="C29" s="92">
-        <f t="shared" ca="1" si="0"/>
+      <c r="A29" s="66"/>
+      <c r="B29" s="76" t="s">
+        <v>136</v>
+      </c>
+      <c r="C29" s="74">
+        <f t="shared" ca="1" si="4"/>
         <v>5</v>
       </c>
-      <c r="D29" s="85">
-        <v>45959</v>
-      </c>
-      <c r="E29" s="71">
+      <c r="D29" s="88">
+        <v>46202</v>
+      </c>
+      <c r="E29" s="65">
         <v>46203</v>
       </c>
-      <c r="F29" s="79">
+      <c r="F29" s="84">
         <v>45960</v>
       </c>
-      <c r="G29" s="78">
-        <v>0</v>
-      </c>
-      <c r="H29" s="82">
+      <c r="G29" s="64">
+        <v>0</v>
+      </c>
+      <c r="H29" s="68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I29" s="68">
+        <f t="shared" si="6"/>
+        <v>100</v>
+      </c>
+      <c r="J29" s="36">
+        <f t="shared" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="K29" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I29" s="82">
+        <v>281</v>
+      </c>
+      <c r="L29" s="37">
         <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="J29" s="38">
-        <f>$J$3</f>
-        <v>45921</v>
-      </c>
-      <c r="K29" s="39">
-        <f>IF(ISBLANK(D29),0,D29-J29)</f>
-        <v>38</v>
-      </c>
-      <c r="L29" s="39">
-        <f>$G29*$O29</f>
-        <v>0</v>
-      </c>
-      <c r="M29" s="39">
+        <v>0</v>
+      </c>
+      <c r="M29" s="37">
         <f>O29-L29</f>
-        <v>244</v>
-      </c>
-      <c r="N29" s="39">
-        <f>IF(ISBLANK(F29),0,(F29-D29)-O29)</f>
+        <v>1</v>
+      </c>
+      <c r="N29" s="101">
+        <f t="shared" si="3"/>
         <v>-243</v>
       </c>
-      <c r="O29" s="40">
-        <f>IF(ISBLANK(E29),0,E29-D29)</f>
-        <v>244</v>
+      <c r="O29" s="99">
+        <f t="shared" si="8"/>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:15" s="11" customFormat="1" ht="46.05" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="25"/>
-      <c r="B30" s="41"/>
-      <c r="C30" s="42"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="44"/>
-      <c r="I30" s="44"/>
-      <c r="J30" s="43"/>
-      <c r="K30" s="45"/>
-      <c r="L30" s="45"/>
-      <c r="M30" s="45"/>
-      <c r="N30" s="45"/>
-      <c r="O30" s="46"/>
+      <c r="B30" s="38"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="39"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="41"/>
+      <c r="I30" s="41"/>
+      <c r="J30" s="40"/>
+      <c r="K30" s="42"/>
+      <c r="L30" s="42"/>
+      <c r="M30" s="42"/>
+      <c r="N30" s="42"/>
+      <c r="O30" s="43"/>
     </row>
     <row r="34" spans="14:14" x14ac:dyDescent="0.2">
       <c r="N34" s="19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G5:I30">
-    <cfRule type="dataBar" priority="7">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="8" tint="0.39997558519241921"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C418AF5D-1E15-4890-9C99-E5C9D08F1B88}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C2:C1048576">
     <cfRule type="colorScale" priority="2">
       <colorScale>
@@ -10125,6 +10292,20 @@
   <conditionalFormatting sqref="C5:C1048576">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Done">
       <formula>NOT(ISERROR(SEARCH("Done",C5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5:I30">
+    <cfRule type="dataBar" priority="7">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color theme="8" tint="0.39997558519241921"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{C418AF5D-1E15-4890-9C99-E5C9D08F1B88}</x14:id>
+        </ext>
+      </extLst>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -10200,13 +10381,13 @@
     </row>
     <row r="7" spans="1:4" ht="15.05" x14ac:dyDescent="0.2">
       <c r="B7" s="18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D7" s="6"/>
     </row>
     <row r="8" spans="1:4" ht="15.05" x14ac:dyDescent="0.2">
       <c r="B8" s="17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D8" s="6"/>
     </row>
@@ -10339,39 +10520,39 @@
   <sheetData>
     <row r="1" spans="1:7" ht="14.85" x14ac:dyDescent="0.2">
       <c r="A1" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="C1" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="D1" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="E1" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="F1" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="G1" s="21" t="s">
         <v>39</v>
-      </c>
-      <c r="F1" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="G1" s="21" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="14.85" x14ac:dyDescent="0.2">
       <c r="A2" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="C2" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="D2" s="22" t="s">
         <v>43</v>
-      </c>
-      <c r="D2" s="22" t="s">
-        <v>44</v>
       </c>
       <c r="E2" s="22">
         <v>2</v>
@@ -10381,19 +10562,19 @@
         <v>14</v>
       </c>
       <c r="G2" s="22" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A3" s="22"/>
       <c r="B3" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="D3" s="22" t="s">
         <v>47</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>48</v>
       </c>
       <c r="E3" s="22">
         <v>3</v>
@@ -10403,19 +10584,19 @@
         <v>21</v>
       </c>
       <c r="G3" s="22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="22"/>
       <c r="B4" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="D4" s="22" t="s">
         <v>51</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>52</v>
       </c>
       <c r="E4" s="22">
         <v>1.5</v>
@@ -10425,21 +10606,21 @@
         <v>11</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="14.85" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="C5" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="D5" s="22" t="s">
         <v>56</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>57</v>
       </c>
       <c r="E5" s="22">
         <v>1.5</v>
@@ -10449,19 +10630,19 @@
         <v>11</v>
       </c>
       <c r="G5" s="22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="22"/>
       <c r="B6" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="22" t="s">
         <v>59</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="22" t="s">
-        <v>60</v>
       </c>
       <c r="E6" s="22">
         <v>4</v>
@@ -10471,19 +10652,19 @@
         <v>28</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="22"/>
       <c r="B7" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="D7" s="22" t="s">
         <v>63</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>64</v>
       </c>
       <c r="E7" s="22">
         <v>2</v>
@@ -10493,19 +10674,19 @@
         <v>14</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="22"/>
       <c r="B8" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="22" t="s">
         <v>66</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>67</v>
       </c>
       <c r="E8" s="22">
         <v>3</v>
@@ -10515,21 +10696,21 @@
         <v>21</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="14.85" x14ac:dyDescent="0.2">
       <c r="A9" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="C9" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="D9" s="22" t="s">
         <v>71</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>72</v>
       </c>
       <c r="E9" s="22">
         <v>1.5</v>
@@ -10539,19 +10720,19 @@
         <v>11</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="22"/>
       <c r="B10" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" s="22" t="s">
         <v>74</v>
-      </c>
-      <c r="C10" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>75</v>
       </c>
       <c r="E10" s="22">
         <v>1.5</v>
@@ -10561,19 +10742,19 @@
         <v>11</v>
       </c>
       <c r="G10" s="22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="22"/>
       <c r="B11" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="D11" s="22" t="s">
         <v>78</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>79</v>
       </c>
       <c r="E11" s="22">
         <v>3</v>
@@ -10583,21 +10764,21 @@
         <v>21</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="14.85" x14ac:dyDescent="0.2">
       <c r="A12" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="C12" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" s="22" t="s">
         <v>82</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="D12" s="22" t="s">
-        <v>83</v>
       </c>
       <c r="E12" s="22">
         <v>2</v>
@@ -10607,19 +10788,19 @@
         <v>14</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="22"/>
       <c r="B13" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="22" t="s">
         <v>85</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="D13" s="22" t="s">
-        <v>86</v>
       </c>
       <c r="E13" s="22">
         <v>2</v>
@@ -10629,19 +10810,19 @@
         <v>14</v>
       </c>
       <c r="G13" s="22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="22"/>
       <c r="B14" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="D14" s="22" t="s">
         <v>88</v>
-      </c>
-      <c r="C14" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" s="22" t="s">
-        <v>89</v>
       </c>
       <c r="E14" s="22">
         <v>3</v>
@@ -10651,19 +10832,19 @@
         <v>21</v>
       </c>
       <c r="G14" s="22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="22"/>
       <c r="B15" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="D15" s="22" t="s">
         <v>92</v>
-      </c>
-      <c r="D15" s="22" t="s">
-        <v>93</v>
       </c>
       <c r="E15" s="22">
         <v>1.5</v>
@@ -10673,21 +10854,21 @@
         <v>11</v>
       </c>
       <c r="G15" s="22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A16" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="22" t="s">
         <v>95</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="C16" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="D16" s="22" t="s">
         <v>97</v>
-      </c>
-      <c r="D16" s="22" t="s">
-        <v>98</v>
       </c>
       <c r="E16" s="22">
         <v>1.5</v>
@@ -10697,19 +10878,19 @@
         <v>11</v>
       </c>
       <c r="G16" s="22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A17" s="22"/>
       <c r="B17" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="D17" s="22" t="s">
         <v>101</v>
-      </c>
-      <c r="D17" s="22" t="s">
-        <v>102</v>
       </c>
       <c r="E17" s="22">
         <v>3</v>
@@ -10719,19 +10900,19 @@
         <v>21</v>
       </c>
       <c r="G17" s="22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="22"/>
       <c r="B18" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="22" t="s">
         <v>104</v>
-      </c>
-      <c r="C18" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="D18" s="22" t="s">
-        <v>105</v>
       </c>
       <c r="E18" s="22">
         <v>3</v>
@@ -10741,21 +10922,21 @@
         <v>21</v>
       </c>
       <c r="G18" s="22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="14.85" x14ac:dyDescent="0.2">
       <c r="A19" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="C19" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" s="22" t="s">
         <v>108</v>
-      </c>
-      <c r="C19" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="D19" s="22" t="s">
-        <v>109</v>
       </c>
       <c r="E19" s="22">
         <v>1.5</v>
@@ -10765,19 +10946,19 @@
         <v>11</v>
       </c>
       <c r="G19" s="22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="22"/>
       <c r="B20" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="C20" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="D20" s="22" t="s">
         <v>112</v>
-      </c>
-      <c r="D20" s="22" t="s">
-        <v>113</v>
       </c>
       <c r="E20" s="22">
         <v>1.5</v>
@@ -10787,21 +10968,21 @@
         <v>11</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="14.85" x14ac:dyDescent="0.2">
       <c r="A21" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="B21" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="C21" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="C21" s="22" t="s">
-        <v>117</v>
-      </c>
       <c r="D21" s="22" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E21" s="22">
         <v>3.5</v>
@@ -10811,19 +10992,19 @@
         <v>25</v>
       </c>
       <c r="G21" s="22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="22"/>
       <c r="B22" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="D22" s="22" t="s">
         <v>119</v>
-      </c>
-      <c r="C22" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>120</v>
       </c>
       <c r="E22" s="22">
         <v>3</v>
@@ -10833,19 +11014,19 @@
         <v>21</v>
       </c>
       <c r="G22" s="22" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="22"/>
       <c r="B23" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="D23" s="22" t="s">
         <v>122</v>
-      </c>
-      <c r="C23" s="22" t="s">
-        <v>113</v>
-      </c>
-      <c r="D23" s="22" t="s">
-        <v>123</v>
       </c>
       <c r="E23" s="22">
         <v>3</v>
@@ -10855,7 +11036,7 @@
         <v>21</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -10879,30 +11060,30 @@
   <sheetData>
     <row r="1" spans="1:8" ht="14.85" x14ac:dyDescent="0.2">
       <c r="A1" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="C1" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="D1" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="21" t="s">
-        <v>38</v>
-      </c>
       <c r="E1" s="21" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="29.7" x14ac:dyDescent="0.2">
       <c r="A2" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="22" t="s">
         <v>41</v>
-      </c>
-      <c r="B2" s="22" t="s">
-        <v>42</v>
       </c>
       <c r="C2" s="24">
         <v>45902</v>
@@ -10914,7 +11095,7 @@
         <v>14</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G2" s="20">
         <f xml:space="preserve"> C2+19</f>
@@ -10928,7 +11109,7 @@
     <row r="3" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A3" s="22"/>
       <c r="B3" s="22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C3" s="24">
         <v>45909</v>
@@ -10940,7 +11121,7 @@
         <v>21</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G3" s="20">
         <f t="shared" ref="G3:G23" si="0" xml:space="preserve"> C3+19</f>
@@ -10954,7 +11135,7 @@
     <row r="4" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A4" s="22"/>
       <c r="B4" s="22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C4" s="24">
         <v>45925</v>
@@ -10966,7 +11147,7 @@
         <v>10</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G4" s="20">
         <f t="shared" si="0"/>
@@ -10979,10 +11160,10 @@
     </row>
     <row r="5" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="22" t="s">
         <v>54</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>55</v>
       </c>
       <c r="C5" s="24">
         <v>45931</v>
@@ -10994,7 +11175,7 @@
         <v>10</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G5" s="20">
         <f t="shared" si="0"/>
@@ -11008,7 +11189,7 @@
     <row r="6" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A6" s="22"/>
       <c r="B6" s="22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C6" s="24">
         <v>45940</v>
@@ -11020,7 +11201,7 @@
         <v>32</v>
       </c>
       <c r="F6" s="22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G6" s="20">
         <f t="shared" si="0"/>
@@ -11034,7 +11215,7 @@
     <row r="7" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A7" s="22"/>
       <c r="B7" s="22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C7" s="24">
         <v>45950</v>
@@ -11046,7 +11227,7 @@
         <v>17</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G7" s="20">
         <f t="shared" si="0"/>
@@ -11060,7 +11241,7 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="22"/>
       <c r="B8" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C8" s="24">
         <v>45966</v>
@@ -11072,7 +11253,7 @@
         <v>20</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G8" s="20">
         <f t="shared" si="0"/>
@@ -11085,10 +11266,10 @@
     </row>
     <row r="9" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A9" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="22" t="s">
         <v>69</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>70</v>
       </c>
       <c r="C9" s="24">
         <v>45992</v>
@@ -11100,7 +11281,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G9" s="20">
         <f t="shared" si="0"/>
@@ -11114,7 +11295,7 @@
     <row r="10" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A10" s="22"/>
       <c r="B10" s="22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C10" s="24">
         <v>46001</v>
@@ -11126,7 +11307,7 @@
         <v>10</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G10" s="20">
         <f t="shared" si="0"/>
@@ -11140,7 +11321,7 @@
     <row r="11" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A11" s="22"/>
       <c r="B11" s="22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C11" s="24">
         <v>46006</v>
@@ -11152,7 +11333,7 @@
         <v>22</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G11" s="20">
         <f t="shared" si="0"/>
@@ -11165,10 +11346,10 @@
     </row>
     <row r="12" spans="1:8" ht="14.85" x14ac:dyDescent="0.2">
       <c r="A12" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" s="22" t="s">
         <v>81</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>82</v>
       </c>
       <c r="C12" s="24">
         <v>46027</v>
@@ -11180,7 +11361,7 @@
         <v>15</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G12" s="20">
         <f t="shared" si="0"/>
@@ -11194,7 +11375,7 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="22"/>
       <c r="B13" s="22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C13" s="24">
         <v>46042</v>
@@ -11206,7 +11387,7 @@
         <v>17</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G13" s="20">
         <f t="shared" si="0"/>
@@ -11220,7 +11401,7 @@
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="22"/>
       <c r="B14" s="22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C14" s="24">
         <v>46058</v>
@@ -11232,7 +11413,7 @@
         <v>21</v>
       </c>
       <c r="F14" s="22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G14" s="20">
         <f t="shared" si="0"/>
@@ -11246,7 +11427,7 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="22"/>
       <c r="B15" s="22" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C15" s="24">
         <v>46073</v>
@@ -11258,7 +11439,7 @@
         <v>10</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G15" s="20">
         <f t="shared" si="0"/>
@@ -11271,10 +11452,10 @@
     </row>
     <row r="16" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A16" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="22" t="s">
         <v>95</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>96</v>
       </c>
       <c r="C16" s="24">
         <v>46082</v>
@@ -11286,7 +11467,7 @@
         <v>10</v>
       </c>
       <c r="F16" s="22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G16" s="20">
         <f t="shared" si="0"/>
@@ -11300,7 +11481,7 @@
     <row r="17" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A17" s="22"/>
       <c r="B17" s="22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C17" s="24">
         <v>46086</v>
@@ -11312,7 +11493,7 @@
         <v>21</v>
       </c>
       <c r="F17" s="22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G17" s="20">
         <f t="shared" si="0"/>
@@ -11326,7 +11507,7 @@
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="22"/>
       <c r="B18" s="22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C18" s="24">
         <v>46091</v>
@@ -11338,7 +11519,7 @@
         <v>21</v>
       </c>
       <c r="F18" s="22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G18" s="20">
         <f t="shared" si="0"/>
@@ -11351,10 +11532,10 @@
     </row>
     <row r="19" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A19" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="22" t="s">
         <v>107</v>
-      </c>
-      <c r="B19" s="22" t="s">
-        <v>108</v>
       </c>
       <c r="C19" s="24">
         <v>46106</v>
@@ -11366,7 +11547,7 @@
         <v>12</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G19" s="20">
         <f t="shared" si="0"/>
@@ -11380,7 +11561,7 @@
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="22"/>
       <c r="B20" s="22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C20" s="24">
         <v>46113</v>
@@ -11392,7 +11573,7 @@
         <v>10</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G20" s="20">
         <f t="shared" si="0"/>
@@ -11405,10 +11586,10 @@
     </row>
     <row r="21" spans="1:8" ht="14.85" x14ac:dyDescent="0.2">
       <c r="A21" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="B21" s="22" t="s">
         <v>115</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>116</v>
       </c>
       <c r="C21" s="24">
         <v>46096</v>
@@ -11420,7 +11601,7 @@
         <v>27</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G21" s="20">
         <f t="shared" si="0"/>
@@ -11434,7 +11615,7 @@
     <row r="22" spans="1:8" ht="28.2" x14ac:dyDescent="0.2">
       <c r="A22" s="22"/>
       <c r="B22" s="22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C22" s="24">
         <v>46106</v>
@@ -11446,7 +11627,7 @@
         <v>22</v>
       </c>
       <c r="F22" s="22" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G22" s="20">
         <f t="shared" si="0"/>
@@ -11460,7 +11641,7 @@
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="22"/>
       <c r="B23" s="22" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C23" s="24">
         <v>46122</v>
@@ -11472,7 +11653,7 @@
         <v>21</v>
       </c>
       <c r="F23" s="22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G23" s="20">
         <f t="shared" si="0"/>
@@ -11497,14 +11678,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="62" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="62" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="74" t="s">
+      <c r="C1" s="62" t="s">
         <v>128</v>
-      </c>
-      <c r="C1" s="74" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>